<commit_message>
test: add multi-line text cases to whitespace trim tests
Add row 2 to both inlineStr and SharedStrings sheets with multi-line
text (containing embedded newlines). Verify that trimming strips
leading/trailing whitespace while preserving inner newlines, and
that xml:space="preserve" opts out of trimming entirely.

Switch from range_eq! macro to individual assert_eq! calls to
accommodate rows with different column counts.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/whitespace_trim.xlsx
+++ b/tests/whitespace_trim.xlsx
@@ -9,7 +9,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>  trimmed value</t>
   </si>
@@ -22,6 +22,14 @@
   </si>
   <si>
     <t>clean text</t>
+  </si>
+  <si>
+    <t>  line1
+line2  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  line1
+line2  </t>
   </si>
 </sst>
 </file>
@@ -87,6 +95,20 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>  line1
+line2  </t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  line1
+line2  </t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -108,6 +130,14 @@
         <v>3</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(xlsx): trim joined <t> text using ASCII whitespace only
Join all text events within <t> before trimming, instead of trimming
each quick-xml Text event separately. This preserves legitimate internal
spaces when XML entities split text across events, while still removing
leading/trailing ASCII whitespace (space/tab/CR/LF only). Also keeps
literal x000D escapes intact during trimming and avoids stripping Unicode
spaces such as U+00A0 (NBSP).
</commit_message>
<xml_diff>
--- a/tests/whitespace_trim.xlsx
+++ b/tests/whitespace_trim.xlsx
@@ -9,7 +9,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>  trimmed value</t>
   </si>
@@ -30,6 +30,9 @@
   <si>
     <t xml:space="preserve">  line1
 line2  </t>
+  </si>
+  <si>
+    <t>日期 时间</t>
   </si>
 </sst>
 </file>
@@ -109,6 +112,13 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>日期 时间</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -138,6 +148,11 @@
         <v>5</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(xlsx): fix whitespace trimming bug introduced in #671 (#673)
* fix(xlsx): trim joined <t> text using ASCII whitespace only

Join all text events within <t> before trimming, instead of trimming
each quick-xml Text event separately. This preserves legitimate internal
spaces when XML entities split text across events, while still removing
leading/trailing ASCII whitespace (space/tab/CR/LF only). Also keeps
literal x000D escapes intact during trimming and avoids stripping Unicode
spaces such as U+00A0 (NBSP).
</commit_message>
<xml_diff>
--- a/tests/whitespace_trim.xlsx
+++ b/tests/whitespace_trim.xlsx
@@ -9,7 +9,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>  trimmed value</t>
   </si>
@@ -30,6 +30,9 @@
   <si>
     <t xml:space="preserve">  line1
 line2  </t>
+  </si>
+  <si>
+    <t>日期 时间</t>
   </si>
 </sst>
 </file>
@@ -109,6 +112,13 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>日期 时间</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -138,6 +148,11 @@
         <v>5</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>